<commit_message>
dodane statistike centilov in con
</commit_message>
<xml_diff>
--- a/reportOKSanaliza.xlsx
+++ b/reportOKSanaliza.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bojan\Documents\GitHub\ReportOKS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A274C62-E0A4-4B79-A1B2-8B961B2310DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63C027AC-76C3-4026-948E-1BA8239ED2DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{8F13620D-0B35-4D77-9205-B40C0C733A79}"/>
   </bookViews>
@@ -22,7 +22,7 @@
   <calcPr calcId="191029"/>
   <pivotCaches>
     <pivotCache cacheId="0" r:id="rId6"/>
-    <pivotCache cacheId="10" r:id="rId7"/>
+    <pivotCache cacheId="1" r:id="rId7"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -56,8 +56,16 @@
 Comment:
     --statistike meritve (centili, cone) ločeno po testu za udeležence OKS projekta Zmigaj_se_do_vadbe (ZV) - regije in SLO
 --BL, 2026-04-01
---centili Slovenija
-SELECT 'Slovenija' as Regija,
+-- definicija baterij kot table variable
+DECLARE @Baterije TABLE (ID INT);
+INSERT INTO @Baterije (ID)
+VALUES (18), (19), (20), (21), (25), (26);
+-- =========================
+-- CENTILI
+-- =========================
+-- centili Slovenija
+SELECT 
+    'Slovenija' as Regija,
     t.Ime AS Test,
     AVG(r.CentilniRang1) AS CentilXA,
     COUNT(r.CentilniRang1) AS N
@@ -69,15 +77,15 @@
 JOIN Merjenec m 
     ON m.ID = r.IdMerjenec
 JOIN Meritev me
-    ON me.ID = m.IdMeritev         -- &lt;--- dodano
+    ON me.ID = m.IdMeritev
 JOIN DostopUporabnikaDoClana du
     ON du.IdClan = m.IdClan
 WHERE du.IdVloga = 10
   AND r.CentilniRang1 IS NOT NULL
-  AND me.BaterijaTestov IN (18, 19, 20, 21, 25, 26)   -- &lt;--- dodan pogoj
+  AND tv.IdBaterija IN (SELECT ID FROM @Baterije)
+  AND me.BaterijaTestov IN (SELECT ID FROM @Baterije)
 GROUP BY 
     t.Ime
---ORDER BY     t.Ime
 UNION ALL
 -- centili regije
 SELECT
@@ -93,7 +101,7 @@
 JOIN Merjenec m 
     ON m.ID = r.IdMerjenec
 JOIN Meritev me
-    ON me.ID = m.IdMeritev     -- &lt;--- dodan povezovalni JOIN
+    ON me.ID = m.IdMeritev
 JOIN DostopUporabnikaDoClana du
     ON du.IdClan = m.IdClan
 JOIN Uporabnik u
@@ -104,14 +112,71 @@
     ON rgn.ID = pc.RegionID
 WHERE du.IdVloga = 10
   AND r.CentilniRang1 IS NOT NULL
-  AND tv.IdBaterija IN (18, 19, 20, 21, 25, 26)    -- testi iz teh baterij
-  AND me.BaterijaTestov IN (18, 19, 20, 21, 25, 26) -- meritve morajo biti v teh baterijah
+  AND tv.IdBaterija IN (SELECT ID FROM @Baterije)
+  AND me.BaterijaTestov IN (SELECT ID FROM @Baterije)
 GROUP BY 
     rgn.Name,
     t.Ime
 ORDER BY 
-    Regija ASC,
-    t.Ime ASC;</t>
+    Regija,
+    Test;
+-- =========================
+-- CONE
+-- =========================
+-- cone Slovenija
+SELECT 
+    'Slovenija' as Regija,
+    te.Ime AS TestIme,
+    SUM(CASE WHEN r.ConaBarva = '#9ac263' THEN 1 ELSE 0 END) AS Zdravo,
+    SUM(CASE WHEN r.ConaBarva = '#ffd54e' THEN 1 ELSE 0 END) AS Mejno,
+    SUM(CASE WHEN r.ConaBarva = '#df3127' THEN 1 ELSE 0 END) AS Tvegano
+FROM Rezultat r
+JOIN Merjenec m 
+    ON m.ID = r.IdMerjenec
+JOIN Meritev me
+    ON me.ID = m.IdMeritev
+JOIN Clan c
+    ON c.ID = m.IdClan
+JOIN Test te
+    ON te.ID = r.IdTest
+WHERE me.BaterijaTestov IN (SELECT ID FROM @Baterije)
+  AND r.ConaBarva IN ('#9ac263', '#df3127', '#ffd54e')
+GROUP BY
+    te.Ime
+UNION ALL
+-- cone regije
+SELECT
+    rgn.Name AS Regija,
+    te.Ime AS TestIme,
+    SUM(CASE WHEN r.ConaBarva = '#9ac263' THEN 1 ELSE 0 END) AS Zdravo,
+    SUM(CASE WHEN r.ConaBarva = '#ffd54e' THEN 1 ELSE 0 END) AS Mejno,
+    SUM(CASE WHEN r.ConaBarva = '#df3127' THEN 1 ELSE 0 END) AS Tvegano
+FROM Rezultat r
+JOIN Merjenec m 
+    ON m.ID = r.IdMerjenec
+JOIN Meritev me
+    ON me.ID = m.IdMeritev
+JOIN Clan c
+    ON c.ID = m.IdClan
+JOIN DostopUporabnikaDoClana du
+    ON du.IdClan = c.ID
+JOIN Uporabnik u
+    ON u.ID = du.IdUporabnik
+JOIN PostalCodes pc
+    ON pc.ID = u.PostalCodeID
+JOIN fitnessMapRegions rgn
+    ON rgn.ID = pc.RegionID
+JOIN Test te
+    ON te.ID = r.IdTest
+WHERE me.BaterijaTestov IN (SELECT ID FROM @Baterije)
+  AND du.IdVloga = 10
+  AND r.ConaBarva IN ('#9ac263', '#ffd54e', '#df3127')
+GROUP BY
+    rgn.Name,
+    te.Ime
+ORDER BY
+    Regija,
+    TestIme;</t>
       </text>
     </comment>
   </commentList>
@@ -129,11 +194,80 @@
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
-    SELECT 'Slovenija' as Regija,
+    -- definicija baterij kot table variable
+DECLARE @Baterije TABLE (ID INT);
+INSERT INTO @Baterije (ID)
+VALUES (18), (19), (20), (21), (25), (26);
+-- =========================
+-- CENTILI
+-- =========================
+-- centili Slovenija
+SELECT 
+    'Slovenija' as Regija,
+    t.Ime AS Test,
+    AVG(r.CentilniRang1) AS CentilXA,
+    COUNT(r.CentilniRang1) AS N
+FROM TestVbateriji tv
+JOIN Test t 
+    ON t.ID = tv.IdTest
+JOIN Rezultat r
+    ON r.IdTest = t.ID
+JOIN Merjenec m 
+    ON m.ID = r.IdMerjenec
+JOIN Meritev me
+    ON me.ID = m.IdMeritev
+JOIN DostopUporabnikaDoClana du
+    ON du.IdClan = m.IdClan
+WHERE du.IdVloga = 10
+  AND r.CentilniRang1 IS NOT NULL
+  AND tv.IdBaterija IN (SELECT ID FROM @Baterije)
+  AND me.BaterijaTestov IN (SELECT ID FROM @Baterije)
+GROUP BY 
+    t.Ime
+UNION ALL
+-- centili regije
+SELECT
+    rgn.Name AS Regija,
+    t.Ime AS Test,
+    AVG(r.CentilniRang1) AS CentilXA,
+    COUNT(r.CentilniRang1) AS N
+FROM TestVbateriji tv
+JOIN Test t 
+    ON t.ID = tv.IdTest
+JOIN Rezultat r
+    ON r.IdTest = t.ID
+JOIN Merjenec m 
+    ON m.ID = r.IdMerjenec
+JOIN Meritev me
+    ON me.ID = m.IdMeritev
+JOIN DostopUporabnikaDoClana du
+    ON du.IdClan = m.IdClan
+JOIN Uporabnik u
+    ON u.ID = du.IdUporabnik
+JOIN PostalCodes pc
+    ON pc.ID = u.PostalCodeID
+JOIN fitnessMapRegions rgn
+    ON rgn.ID = pc.RegionID
+WHERE du.IdVloga = 10
+  AND r.CentilniRang1 IS NOT NULL
+  AND tv.IdBaterija IN (SELECT ID FROM @Baterije)
+  AND me.BaterijaTestov IN (SELECT ID FROM @Baterije)
+GROUP BY 
+    rgn.Name,
+    t.Ime
+ORDER BY 
+    Regija,
+    Test;
+-- =========================
+-- CONE
+-- =========================
+-- cone Slovenija
+SELECT 
+    'Slovenija' as Regija,
     te.Ime AS TestIme,
-    SUM(CASE WHEN r.ConaBarva = '#9ac263' THEN 1 ELSE 0 END) AS Zdravo,   -- zelena
-    SUM(CASE WHEN r.ConaBarva = '#ffd54e' THEN 1 ELSE 0 END) AS Mejno,    -- rumena
-    SUM(CASE WHEN r.ConaBarva = '#df3127' THEN 1 ELSE 0 END) AS Tvegano   -- rdeča
+    SUM(CASE WHEN r.ConaBarva = '#9ac263' THEN 1 ELSE 0 END) AS Zdravo,
+    SUM(CASE WHEN r.ConaBarva = '#ffd54e' THEN 1 ELSE 0 END) AS Mejno,
+    SUM(CASE WHEN r.ConaBarva = '#df3127' THEN 1 ELSE 0 END) AS Tvegano
 FROM Rezultat r
 JOIN Merjenec m 
     ON m.ID = r.IdMerjenec
@@ -143,18 +277,18 @@
     ON c.ID = m.IdClan
 JOIN Test te
     ON te.ID = r.IdTest
-WHERE me.BaterijaTestov IN (18, 19, 20, 21, 25, 26)
+WHERE me.BaterijaTestov IN (SELECT ID FROM @Baterije)
   AND r.ConaBarva IN ('#9ac263', '#df3127', '#ffd54e')
 GROUP BY
     te.Ime
---ORDER BY     te.Ime
 UNION ALL
+-- cone regije
 SELECT
     rgn.Name AS Regija,
     te.Ime AS TestIme,
-    SUM(CASE WHEN r.ConaBarva = '#9ac263' THEN 1 ELSE 0 END) AS Zdravo,   -- zelena
-    SUM(CASE WHEN r.ConaBarva = '#ffd54e' THEN 1 ELSE 0 END) AS Mejno,    -- rumena
-    SUM(CASE WHEN r.ConaBarva = '#df3127' THEN 1 ELSE 0 END) AS Tvegano   -- rdeča
+    SUM(CASE WHEN r.ConaBarva = '#9ac263' THEN 1 ELSE 0 END) AS Zdravo,
+    SUM(CASE WHEN r.ConaBarva = '#ffd54e' THEN 1 ELSE 0 END) AS Mejno,
+    SUM(CASE WHEN r.ConaBarva = '#df3127' THEN 1 ELSE 0 END) AS Tvegano
 FROM Rezultat r
 JOIN Merjenec m 
     ON m.ID = r.IdMerjenec
@@ -172,15 +306,15 @@
     ON rgn.ID = pc.RegionID
 JOIN Test te
     ON te.ID = r.IdTest
-WHERE me.BaterijaTestov IN (18, 19, 20, 21, 25, 26)
+WHERE me.BaterijaTestov IN (SELECT ID FROM @Baterije)
   AND du.IdVloga = 10
   AND r.ConaBarva IN ('#9ac263', '#ffd54e', '#df3127')
 GROUP BY
     rgn.Name,
     te.Ime
 ORDER BY
-    Regija ASC,
-    te.Ime ASC;</t>
+    Regija,
+    TestIme;</t>
       </text>
     </comment>
   </commentList>
@@ -1838,7 +1972,7 @@
     <numFmt numFmtId="164" formatCode="0.0"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1863,12 +1997,6 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
-      <charset val="1"/>
     </font>
   </fonts>
   <fills count="4">
@@ -1920,7 +2048,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
@@ -1931,7 +2059,6 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="3">
@@ -1939,16 +2066,7 @@
     <cellStyle name="Normal 2" xfId="1" xr:uid="{BDBFD1E4-62EC-41BE-B39B-390F134CCF6B}"/>
     <cellStyle name="Percent" xfId="2" builtinId="5"/>
   </cellStyles>
-  <dxfs count="4">
-    <dxf>
-      <numFmt numFmtId="165" formatCode="0.0%"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="165" formatCode="0.0%"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="13" formatCode="0%"/>
-    </dxf>
+  <dxfs count="1">
     <dxf>
       <numFmt numFmtId="165" formatCode="0.0%"/>
     </dxf>
@@ -4476,8 +4594,8 @@
     <xdr:to>
       <xdr:col>18</xdr:col>
       <xdr:colOff>266700</xdr:colOff>
-      <xdr:row>37</xdr:row>
-      <xdr:rowOff>137160</xdr:rowOff>
+      <xdr:row>40</xdr:row>
+      <xdr:rowOff>167640</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -7361,7 +7479,7 @@
     <dataField name="Average of CentilXA" fld="2" subtotal="average" baseField="0" baseItem="0" numFmtId="164"/>
   </dataFields>
   <conditionalFormats count="2">
-    <conditionalFormat priority="1">
+    <conditionalFormat priority="3">
       <pivotAreas count="1">
         <pivotArea type="data" collapsedLevelsAreSubtotals="1" fieldPosition="0">
           <references count="2">
@@ -7387,7 +7505,7 @@
         </pivotArea>
       </pivotAreas>
     </conditionalFormat>
-    <conditionalFormat priority="3">
+    <conditionalFormat priority="1">
       <pivotAreas count="1">
         <pivotArea type="data" collapsedLevelsAreSubtotals="1" fieldPosition="0">
           <references count="2">
@@ -7450,7 +7568,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{ED1F8AC9-8CC5-4E08-995C-C481136EF10E}" name="PivotTable1" cacheId="10" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="5">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{ED1F8AC9-8CC5-4E08-995C-C481136EF10E}" name="PivotTable1" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="5">
   <location ref="K4:M18" firstHeaderRow="0" firstDataRow="1" firstDataCol="1" rowPageCount="1" colPageCount="1"/>
   <pivotFields count="9">
     <pivotField axis="axisRow" showAll="0">
@@ -7561,7 +7679,7 @@
     <dataField name="Average of Mejno%" fld="7" subtotal="average" baseField="0" baseItem="0"/>
   </dataFields>
   <formats count="1">
-    <format dxfId="3">
+    <format dxfId="0">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="0" count="0"/>
@@ -7933,8 +8051,16 @@
   <threadedComment ref="A1" dT="2026-04-03T04:11:08.84" personId="{B0A86080-3FF1-41DA-B9EB-1C8139C00CC1}" id="{F4841313-2AC6-4AB8-9D8D-A918BDBEDA73}">
     <text>--statistike meritve (centili, cone) ločeno po testu za udeležence OKS projekta Zmigaj_se_do_vadbe (ZV) - regije in SLO
 --BL, 2026-04-01
---centili Slovenija
-SELECT 'Slovenija' as Regija,
+-- definicija baterij kot table variable
+DECLARE @Baterije TABLE (ID INT);
+INSERT INTO @Baterije (ID)
+VALUES (18), (19), (20), (21), (25), (26);
+-- =========================
+-- CENTILI
+-- =========================
+-- centili Slovenija
+SELECT 
+    'Slovenija' as Regija,
     t.Ime AS Test,
     AVG(r.CentilniRang1) AS CentilXA,
     COUNT(r.CentilniRang1) AS N
@@ -7946,15 +8072,15 @@
 JOIN Merjenec m 
     ON m.ID = r.IdMerjenec
 JOIN Meritev me
-    ON me.ID = m.IdMeritev         -- &lt;--- dodano
+    ON me.ID = m.IdMeritev
 JOIN DostopUporabnikaDoClana du
     ON du.IdClan = m.IdClan
 WHERE du.IdVloga = 10
   AND r.CentilniRang1 IS NOT NULL
-  AND me.BaterijaTestov IN (18, 19, 20, 21, 25, 26)   -- &lt;--- dodan pogoj
+  AND tv.IdBaterija IN (SELECT ID FROM @Baterije)
+  AND me.BaterijaTestov IN (SELECT ID FROM @Baterije)
 GROUP BY 
     t.Ime
---ORDER BY     t.Ime
 UNION ALL
 -- centili regije
 SELECT
@@ -7970,7 +8096,7 @@
 JOIN Merjenec m 
     ON m.ID = r.IdMerjenec
 JOIN Meritev me
-    ON me.ID = m.IdMeritev     -- &lt;--- dodan povezovalni JOIN
+    ON me.ID = m.IdMeritev
 JOIN DostopUporabnikaDoClana du
     ON du.IdClan = m.IdClan
 JOIN Uporabnik u
@@ -7981,26 +8107,24 @@
     ON rgn.ID = pc.RegionID
 WHERE du.IdVloga = 10
   AND r.CentilniRang1 IS NOT NULL
-  AND tv.IdBaterija IN (18, 19, 20, 21, 25, 26)    -- testi iz teh baterij
-  AND me.BaterijaTestov IN (18, 19, 20, 21, 25, 26) -- meritve morajo biti v teh baterijah
+  AND tv.IdBaterija IN (SELECT ID FROM @Baterije)
+  AND me.BaterijaTestov IN (SELECT ID FROM @Baterije)
 GROUP BY 
     rgn.Name,
     t.Ime
 ORDER BY 
-    Regija ASC,
-    t.Ime ASC;</text>
-  </threadedComment>
-</ThreadedComments>
-</file>
-
-<file path=xl/threadedComments/threadedComment2.xml><?xml version="1.0" encoding="utf-8"?>
-<ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <threadedComment ref="A1" dT="2026-04-03T05:49:55.82" personId="{B0A86080-3FF1-41DA-B9EB-1C8139C00CC1}" id="{BFFC901B-821E-4A6C-8204-68AA98345E97}">
-    <text>SELECT 'Slovenija' as Regija,
+    Regija,
+    Test;
+-- =========================
+-- CONE
+-- =========================
+-- cone Slovenija
+SELECT 
+    'Slovenija' as Regija,
     te.Ime AS TestIme,
-    SUM(CASE WHEN r.ConaBarva = '#9ac263' THEN 1 ELSE 0 END) AS Zdravo,   -- zelena
-    SUM(CASE WHEN r.ConaBarva = '#ffd54e' THEN 1 ELSE 0 END) AS Mejno,    -- rumena
-    SUM(CASE WHEN r.ConaBarva = '#df3127' THEN 1 ELSE 0 END) AS Tvegano   -- rdeča
+    SUM(CASE WHEN r.ConaBarva = '#9ac263' THEN 1 ELSE 0 END) AS Zdravo,
+    SUM(CASE WHEN r.ConaBarva = '#ffd54e' THEN 1 ELSE 0 END) AS Mejno,
+    SUM(CASE WHEN r.ConaBarva = '#df3127' THEN 1 ELSE 0 END) AS Tvegano
 FROM Rezultat r
 JOIN Merjenec m 
     ON m.ID = r.IdMerjenec
@@ -8010,18 +8134,18 @@
     ON c.ID = m.IdClan
 JOIN Test te
     ON te.ID = r.IdTest
-WHERE me.BaterijaTestov IN (18, 19, 20, 21, 25, 26)
+WHERE me.BaterijaTestov IN (SELECT ID FROM @Baterije)
   AND r.ConaBarva IN ('#9ac263', '#df3127', '#ffd54e')
 GROUP BY
     te.Ime
---ORDER BY     te.Ime
 UNION ALL
+-- cone regije
 SELECT
     rgn.Name AS Regija,
     te.Ime AS TestIme,
-    SUM(CASE WHEN r.ConaBarva = '#9ac263' THEN 1 ELSE 0 END) AS Zdravo,   -- zelena
-    SUM(CASE WHEN r.ConaBarva = '#ffd54e' THEN 1 ELSE 0 END) AS Mejno,    -- rumena
-    SUM(CASE WHEN r.ConaBarva = '#df3127' THEN 1 ELSE 0 END) AS Tvegano   -- rdeča
+    SUM(CASE WHEN r.ConaBarva = '#9ac263' THEN 1 ELSE 0 END) AS Zdravo,
+    SUM(CASE WHEN r.ConaBarva = '#ffd54e' THEN 1 ELSE 0 END) AS Mejno,
+    SUM(CASE WHEN r.ConaBarva = '#df3127' THEN 1 ELSE 0 END) AS Tvegano
 FROM Rezultat r
 JOIN Merjenec m 
     ON m.ID = r.IdMerjenec
@@ -8039,15 +8163,143 @@
     ON rgn.ID = pc.RegionID
 JOIN Test te
     ON te.ID = r.IdTest
-WHERE me.BaterijaTestov IN (18, 19, 20, 21, 25, 26)
+WHERE me.BaterijaTestov IN (SELECT ID FROM @Baterije)
   AND du.IdVloga = 10
   AND r.ConaBarva IN ('#9ac263', '#ffd54e', '#df3127')
 GROUP BY
     rgn.Name,
     te.Ime
 ORDER BY
-    Regija ASC,
-    te.Ime ASC;</text>
+    Regija,
+    TestIme;</text>
+  </threadedComment>
+</ThreadedComments>
+</file>
+
+<file path=xl/threadedComments/threadedComment2.xml><?xml version="1.0" encoding="utf-8"?>
+<ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <threadedComment ref="A1" dT="2026-04-03T05:49:55.82" personId="{B0A86080-3FF1-41DA-B9EB-1C8139C00CC1}" id="{BFFC901B-821E-4A6C-8204-68AA98345E97}">
+    <text>-- definicija baterij kot table variable
+DECLARE @Baterije TABLE (ID INT);
+INSERT INTO @Baterije (ID)
+VALUES (18), (19), (20), (21), (25), (26);
+-- =========================
+-- CENTILI
+-- =========================
+-- centili Slovenija
+SELECT 
+    'Slovenija' as Regija,
+    t.Ime AS Test,
+    AVG(r.CentilniRang1) AS CentilXA,
+    COUNT(r.CentilniRang1) AS N
+FROM TestVbateriji tv
+JOIN Test t 
+    ON t.ID = tv.IdTest
+JOIN Rezultat r
+    ON r.IdTest = t.ID
+JOIN Merjenec m 
+    ON m.ID = r.IdMerjenec
+JOIN Meritev me
+    ON me.ID = m.IdMeritev
+JOIN DostopUporabnikaDoClana du
+    ON du.IdClan = m.IdClan
+WHERE du.IdVloga = 10
+  AND r.CentilniRang1 IS NOT NULL
+  AND tv.IdBaterija IN (SELECT ID FROM @Baterije)
+  AND me.BaterijaTestov IN (SELECT ID FROM @Baterije)
+GROUP BY 
+    t.Ime
+UNION ALL
+-- centili regije
+SELECT
+    rgn.Name AS Regija,
+    t.Ime AS Test,
+    AVG(r.CentilniRang1) AS CentilXA,
+    COUNT(r.CentilniRang1) AS N
+FROM TestVbateriji tv
+JOIN Test t 
+    ON t.ID = tv.IdTest
+JOIN Rezultat r
+    ON r.IdTest = t.ID
+JOIN Merjenec m 
+    ON m.ID = r.IdMerjenec
+JOIN Meritev me
+    ON me.ID = m.IdMeritev
+JOIN DostopUporabnikaDoClana du
+    ON du.IdClan = m.IdClan
+JOIN Uporabnik u
+    ON u.ID = du.IdUporabnik
+JOIN PostalCodes pc
+    ON pc.ID = u.PostalCodeID
+JOIN fitnessMapRegions rgn
+    ON rgn.ID = pc.RegionID
+WHERE du.IdVloga = 10
+  AND r.CentilniRang1 IS NOT NULL
+  AND tv.IdBaterija IN (SELECT ID FROM @Baterije)
+  AND me.BaterijaTestov IN (SELECT ID FROM @Baterije)
+GROUP BY 
+    rgn.Name,
+    t.Ime
+ORDER BY 
+    Regija,
+    Test;
+-- =========================
+-- CONE
+-- =========================
+-- cone Slovenija
+SELECT 
+    'Slovenija' as Regija,
+    te.Ime AS TestIme,
+    SUM(CASE WHEN r.ConaBarva = '#9ac263' THEN 1 ELSE 0 END) AS Zdravo,
+    SUM(CASE WHEN r.ConaBarva = '#ffd54e' THEN 1 ELSE 0 END) AS Mejno,
+    SUM(CASE WHEN r.ConaBarva = '#df3127' THEN 1 ELSE 0 END) AS Tvegano
+FROM Rezultat r
+JOIN Merjenec m 
+    ON m.ID = r.IdMerjenec
+JOIN Meritev me
+    ON me.ID = m.IdMeritev
+JOIN Clan c
+    ON c.ID = m.IdClan
+JOIN Test te
+    ON te.ID = r.IdTest
+WHERE me.BaterijaTestov IN (SELECT ID FROM @Baterije)
+  AND r.ConaBarva IN ('#9ac263', '#df3127', '#ffd54e')
+GROUP BY
+    te.Ime
+UNION ALL
+-- cone regije
+SELECT
+    rgn.Name AS Regija,
+    te.Ime AS TestIme,
+    SUM(CASE WHEN r.ConaBarva = '#9ac263' THEN 1 ELSE 0 END) AS Zdravo,
+    SUM(CASE WHEN r.ConaBarva = '#ffd54e' THEN 1 ELSE 0 END) AS Mejno,
+    SUM(CASE WHEN r.ConaBarva = '#df3127' THEN 1 ELSE 0 END) AS Tvegano
+FROM Rezultat r
+JOIN Merjenec m 
+    ON m.ID = r.IdMerjenec
+JOIN Meritev me
+    ON me.ID = m.IdMeritev
+JOIN Clan c
+    ON c.ID = m.IdClan
+JOIN DostopUporabnikaDoClana du
+    ON du.IdClan = c.ID
+JOIN Uporabnik u
+    ON u.ID = du.IdUporabnik
+JOIN PostalCodes pc
+    ON pc.ID = u.PostalCodeID
+JOIN fitnessMapRegions rgn
+    ON rgn.ID = pc.RegionID
+JOIN Test te
+    ON te.ID = r.IdTest
+WHERE me.BaterijaTestov IN (SELECT ID FROM @Baterije)
+  AND du.IdVloga = 10
+  AND r.ConaBarva IN ('#9ac263', '#ffd54e', '#df3127')
+GROUP BY
+    rgn.Name,
+    te.Ime
+ORDER BY
+    Regija,
+    TestIme;</text>
   </threadedComment>
 </ThreadedComments>
 </file>
@@ -10886,10 +11138,10 @@
       <c r="K5" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="L5" s="9">
+      <c r="L5" s="8">
         <v>0.1864406779661017</v>
       </c>
-      <c r="M5" s="9">
+      <c r="M5" s="8">
         <v>0.16949152542372881</v>
       </c>
     </row>
@@ -10928,10 +11180,10 @@
       <c r="K6" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="L6" s="9">
+      <c r="L6" s="8">
         <v>0.21794871794871795</v>
       </c>
-      <c r="M6" s="9">
+      <c r="M6" s="8">
         <v>0.17948717948717949</v>
       </c>
     </row>
@@ -10970,10 +11222,10 @@
       <c r="K7" s="6" t="s">
         <v>96</v>
       </c>
-      <c r="L7" s="9">
+      <c r="L7" s="8">
         <v>0.25490196078431371</v>
       </c>
-      <c r="M7" s="9">
+      <c r="M7" s="8">
         <v>0.14705882352941177</v>
       </c>
     </row>
@@ -11012,10 +11264,10 @@
       <c r="K8" s="6" t="s">
         <v>143</v>
       </c>
-      <c r="L8" s="9">
+      <c r="L8" s="8">
         <v>0.39473684210526316</v>
       </c>
-      <c r="M8" s="9">
+      <c r="M8" s="8">
         <v>0.15789473684210525</v>
       </c>
     </row>
@@ -11054,10 +11306,10 @@
       <c r="K9" s="6" t="s">
         <v>163</v>
       </c>
-      <c r="L9" s="9">
+      <c r="L9" s="8">
         <v>0.32307692307692309</v>
       </c>
-      <c r="M9" s="9">
+      <c r="M9" s="8">
         <v>9.2307692307692313E-2</v>
       </c>
     </row>
@@ -11096,10 +11348,10 @@
       <c r="K10" s="6" t="s">
         <v>191</v>
       </c>
-      <c r="L10" s="9">
+      <c r="L10" s="8">
         <v>0.24878048780487805</v>
       </c>
-      <c r="M10" s="9">
+      <c r="M10" s="8">
         <v>0.2032520325203252</v>
       </c>
     </row>
@@ -11138,10 +11390,10 @@
       <c r="K11" s="6" t="s">
         <v>253</v>
       </c>
-      <c r="L11" s="9">
+      <c r="L11" s="8">
         <v>0.14516129032258066</v>
       </c>
-      <c r="M11" s="9">
+      <c r="M11" s="8">
         <v>0.19354838709677419</v>
       </c>
     </row>
@@ -11180,10 +11432,10 @@
       <c r="K12" s="6" t="s">
         <v>333</v>
       </c>
-      <c r="L12" s="9">
+      <c r="L12" s="8">
         <v>0.23684210526315788</v>
       </c>
-      <c r="M12" s="9">
+      <c r="M12" s="8">
         <v>0.21052631578947367</v>
       </c>
     </row>
@@ -11222,10 +11474,10 @@
       <c r="K13" s="6" t="s">
         <v>371</v>
       </c>
-      <c r="L13" s="9">
+      <c r="L13" s="8">
         <v>0.19379844961240311</v>
       </c>
-      <c r="M13" s="9">
+      <c r="M13" s="8">
         <v>0.27906976744186046</v>
       </c>
     </row>
@@ -11264,10 +11516,10 @@
       <c r="K14" s="6" t="s">
         <v>402</v>
       </c>
-      <c r="L14" s="9">
+      <c r="L14" s="8">
         <v>0.14285714285714285</v>
       </c>
-      <c r="M14" s="9">
+      <c r="M14" s="8">
         <v>0.14285714285714285</v>
       </c>
     </row>
@@ -11306,10 +11558,10 @@
       <c r="K15" s="6" t="s">
         <v>420</v>
       </c>
-      <c r="L15" s="9">
+      <c r="L15" s="8">
         <v>0.203125</v>
       </c>
-      <c r="M15" s="9">
+      <c r="M15" s="8">
         <v>0.2109375</v>
       </c>
     </row>
@@ -11348,10 +11600,10 @@
       <c r="K16" s="6" t="s">
         <v>505</v>
       </c>
-      <c r="L16" s="9">
+      <c r="L16" s="8">
         <v>0.24783974862529459</v>
       </c>
-      <c r="M16" s="9">
+      <c r="M16" s="8">
         <v>0.19285153181461115</v>
       </c>
     </row>
@@ -11390,10 +11642,10 @@
       <c r="K17" s="6" t="s">
         <v>491</v>
       </c>
-      <c r="L17" s="9">
+      <c r="L17" s="8">
         <v>0.22727272727272727</v>
       </c>
-      <c r="M17" s="9">
+      <c r="M17" s="8">
         <v>0.31818181818181818</v>
       </c>
     </row>
@@ -11432,10 +11684,10 @@
       <c r="K18" s="6" t="s">
         <v>531</v>
       </c>
-      <c r="L18" s="8">
+      <c r="L18">
         <v>0.23252169797226951</v>
       </c>
-      <c r="M18" s="8">
+      <c r="M18">
         <v>0.19211265025324029</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Spremenil slog za 2. tabelo, da bo isti kot pri 1.
</commit_message>
<xml_diff>
--- a/reportOKSanaliza.xlsx
+++ b/reportOKSanaliza.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30006"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30019"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bojan\Documents\GitHub\ReportOKS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A7F521F1-22C6-457D-9708-53B651198F90}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{1A7ADBF7-FEED-4078-9ABB-B0F197399286}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="5" xr2:uid="{8F13620D-0B35-4D77-9205-B40C0C733A79}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{8F13620D-0B35-4D77-9205-B40C0C733A79}"/>
   </bookViews>
   <sheets>
     <sheet name="Analize" sheetId="4" r:id="rId1"/>
@@ -22,8 +22,8 @@
   </sheets>
   <calcPr calcId="191028"/>
   <pivotCaches>
-    <pivotCache cacheId="8" r:id="rId7"/>
-    <pivotCache cacheId="9" r:id="rId8"/>
+    <pivotCache cacheId="360" r:id="rId7"/>
+    <pivotCache cacheId="361" r:id="rId8"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -384,7 +384,7 @@
     <t>FŠ odrasli 13.2.2026</t>
   </si>
   <si>
-    <t>Table Grid</t>
+    <t>Light Shading Accent 3</t>
   </si>
   <si>
     <t>Geo_enota</t>
@@ -2099,9 +2099,9 @@
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="3">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Navadno" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 2" xfId="1" xr:uid="{BDBFD1E4-62EC-41BE-B39B-390F134CCF6B}"/>
-    <cellStyle name="Percent" xfId="2" builtinId="5"/>
+    <cellStyle name="Odstotek" xfId="2" builtinId="5"/>
   </cellStyles>
   <dxfs count="1">
     <dxf>
@@ -2123,7 +2123,7 @@
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="en-US"/>
+  <c:lang val="sl-SI"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -2265,7 +2265,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>Total</c:v>
+                  <c:v>Vsota</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -2703,7 +2703,7 @@
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="en-US"/>
+  <c:lang val="sl-SI"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -7408,7 +7408,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{2F335978-D2AF-46A9-AAAA-E269CFBBC0BA}" name="PivotTable1" cacheId="8" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="5">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{2F335978-D2AF-46A9-AAAA-E269CFBBC0BA}" name="PivotTable1" cacheId="360" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="5">
   <location ref="H4:I18" firstHeaderRow="1" firstDataRow="1" firstDataCol="1" rowPageCount="1" colPageCount="1"/>
   <pivotFields count="4">
     <pivotField axis="axisRow" showAll="0">
@@ -7516,7 +7516,7 @@
     <dataField name="Average of CentilXA" fld="2" subtotal="average" baseField="0" baseItem="0" numFmtId="164"/>
   </dataFields>
   <conditionalFormats count="2">
-    <conditionalFormat priority="3">
+    <conditionalFormat priority="1">
       <pivotAreas count="1">
         <pivotArea type="data" collapsedLevelsAreSubtotals="1" fieldPosition="0">
           <references count="2">
@@ -7542,7 +7542,7 @@
         </pivotArea>
       </pivotAreas>
     </conditionalFormat>
-    <conditionalFormat priority="1">
+    <conditionalFormat priority="3">
       <pivotAreas count="1">
         <pivotArea type="data" collapsedLevelsAreSubtotals="1" fieldPosition="0">
           <references count="2">
@@ -7605,7 +7605,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{ED1F8AC9-8CC5-4E08-995C-C481136EF10E}" name="PivotTable1" cacheId="9" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="5">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{ED1F8AC9-8CC5-4E08-995C-C481136EF10E}" name="PivotTable1" cacheId="361" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="5">
   <location ref="K4:M18" firstHeaderRow="0" firstDataRow="1" firstDataCol="1" rowPageCount="1" colPageCount="1"/>
   <pivotFields count="9">
     <pivotField axis="axisRow" showAll="0">
@@ -8368,7 +8368,7 @@
     <col min="1" max="1" width="4.7109375" customWidth="1"/>
     <col min="4" max="4" width="16.42578125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="17.42578125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="20.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6">

</xml_diff>